<commit_message>
New Customs notification mai non-tariff new notification
</commit_message>
<xml_diff>
--- a/backend/PDF_DOC/CBIC/Notifications/Non-Tariff/Non-Tariff Notifications.xlsx
+++ b/backend/PDF_DOC/CBIC/Notifications/Non-Tariff/Non-Tariff Notifications.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9309DCE2-FA9B-4FBE-B9AD-63EB6463261D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C81650BE-AC01-4C7E-B092-2CCF128D185C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="375">
   <si>
     <t>Non-Tariff Notifications : 2024</t>
   </si>
@@ -1141,6 +1141,12 @@
   </si>
   <si>
     <t>63/2026-Customs (N.T)</t>
+  </si>
+  <si>
+    <t>66/2026-Customs (NT)</t>
+  </si>
+  <si>
+    <t>Notification of Udangudi port u/s. 7(1)(a) of Customs Act, 1962" and it was issued under Section 7(1)(a) of Customs Act, 1962.</t>
   </si>
 </sst>
 </file>
@@ -1526,7 +1532,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" customWidth="1"/>
@@ -1562,208 +1568,208 @@
     </row>
     <row r="6" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="B6" s="18">
+        <v>46223</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>369</v>
-      </c>
-      <c r="B6" s="18">
-        <v>46219</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>371</v>
       </c>
       <c r="B7" s="18">
         <v>46219</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="B8" s="18">
+        <v>46219</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>372</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B9" s="3">
         <v>46218</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+      <c r="C9" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" s="14" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="17" t="s">
         <v>367</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B10" s="16">
         <v>46206</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C10" s="15" t="s">
         <v>368</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
-        <v>365</v>
-      </c>
-      <c r="B10" s="12">
-        <v>46204</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
+        <v>365</v>
+      </c>
+      <c r="B11" s="12">
+        <v>46204</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
         <v>364</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B12" s="12">
         <v>46203</v>
       </c>
-      <c r="C11" s="13" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>363</v>
-      </c>
-      <c r="B12" s="9">
-        <v>46202</v>
-      </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="13" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B13" s="9">
-        <v>46195</v>
+        <v>46202</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>357</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B14" s="9">
-        <v>46191</v>
+        <v>46195</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B15" s="9">
-        <v>46189</v>
+        <v>46191</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B16" s="9">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>154</v>
+        <v>353</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="B17" s="9">
+        <v>46188</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
         <v>354</v>
-      </c>
-      <c r="B17" s="9">
-        <v>46184</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>362</v>
       </c>
       <c r="B18" s="9">
         <v>46184</v>
       </c>
       <c r="C18" s="10" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>362</v>
+      </c>
+      <c r="B19" s="9">
+        <v>46184</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>355</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
-        <v>351</v>
-      </c>
-      <c r="B19" s="9">
-        <v>46182</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="B20" s="9">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B21" s="9">
         <v>46178</v>
       </c>
       <c r="C21" s="10" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>344</v>
+      </c>
+      <c r="B22" s="9">
+        <v>46178</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>345</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>346</v>
-      </c>
-      <c r="B22" s="3">
-        <v>46171</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B23" s="3">
-        <v>46161</v>
+        <v>46171</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B24" s="3">
-        <v>46157</v>
+        <v>46161</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>154</v>
@@ -1771,10 +1777,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B25" s="3">
-        <v>46150</v>
+        <v>46157</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>154</v>
@@ -1782,208 +1788,208 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B26" s="3">
-        <v>46148</v>
+        <v>46150</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>341</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>320</v>
+        <v>350</v>
       </c>
       <c r="B27" s="3">
-        <v>46142</v>
+        <v>46148</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>154</v>
+        <v>341</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B28" s="3">
-        <v>46136</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>163</v>
+        <v>46142</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>318</v>
+      </c>
+      <c r="B29" s="3">
+        <v>46136</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>321</v>
       </c>
-      <c r="B29" s="3">
+      <c r="B30" s="3">
         <v>46132</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C30" s="7" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>316</v>
       </c>
-      <c r="B30" s="3">
+      <c r="B31" s="3">
         <v>46128</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>317</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>322</v>
-      </c>
-      <c r="B31" s="3">
-        <v>46127</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B32" s="3">
-        <v>46118</v>
+        <v>46127</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>315</v>
+        <v>154</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B33" s="3">
-        <v>46114</v>
+        <v>46118</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>154</v>
+        <v>315</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>191</v>
+        <v>324</v>
       </c>
       <c r="B34" s="3">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>311</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B35" s="3">
         <v>46112</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>325</v>
+        <v>192</v>
       </c>
       <c r="B36" s="3">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>171</v>
+        <v>312</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B37" s="3">
         <v>46111</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>313</v>
+        <v>171</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B38" s="3">
-        <v>46105</v>
+        <v>46111</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B39" s="3">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B40" s="3">
         <v>46101</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>171</v>
+        <v>309</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B41" s="3">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>265</v>
+        <v>330</v>
       </c>
       <c r="B42" s="3">
-        <v>46097</v>
+        <v>46100</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>310</v>
+        <v>154</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B43" s="3">
-        <v>46094</v>
+        <v>46097</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>154</v>
+        <v>310</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>201</v>
+        <v>266</v>
       </c>
       <c r="B44" s="3">
-        <v>46077</v>
+        <v>46094</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>154</v>
@@ -1991,43 +1997,43 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>201</v>
+      </c>
+      <c r="B45" s="3">
+        <v>46077</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>303</v>
       </c>
-      <c r="B45" s="3">
+      <c r="B46" s="3">
         <v>46071</v>
       </c>
-      <c r="C45" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="C46" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>304</v>
       </c>
-      <c r="B46" s="3">
+      <c r="B47" s="3">
         <v>46069</v>
       </c>
-      <c r="C46" s="2" t="s">
+      <c r="C47" s="2" t="s">
         <v>176</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>305</v>
-      </c>
-      <c r="B47" s="3">
-        <v>46066</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B48" s="3">
-        <v>46059</v>
+        <v>46066</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>154</v>
@@ -2035,10 +2041,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B49" s="3">
-        <v>46058</v>
+        <v>46059</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>154</v>
@@ -2046,98 +2052,98 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>307</v>
+      </c>
+      <c r="B50" s="3">
+        <v>46058</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>308</v>
-      </c>
-      <c r="B50" s="3">
-        <v>46056</v>
-      </c>
-      <c r="C50" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" ht="45" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="s">
-        <v>286</v>
       </c>
       <c r="B51" s="3">
         <v>46056</v>
       </c>
       <c r="C51" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>287</v>
-      </c>
       <c r="B52" s="3">
-        <v>46055</v>
+        <v>46056</v>
       </c>
       <c r="C52" t="s">
-        <v>154</v>
+        <v>286</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B53" s="3">
-        <v>46054</v>
+        <v>46055</v>
       </c>
       <c r="C53" t="s">
-        <v>289</v>
+        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B54" s="3">
         <v>46054</v>
       </c>
       <c r="C54" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B55" s="3">
         <v>46054</v>
       </c>
       <c r="C55" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B56" s="3">
         <v>46054</v>
       </c>
       <c r="C56" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B57" s="3">
-        <v>46052</v>
+        <v>46054</v>
       </c>
       <c r="C57" t="s">
-        <v>154</v>
+        <v>295</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>331</v>
+        <v>296</v>
       </c>
       <c r="B58" s="3">
-        <v>46051</v>
+        <v>46052</v>
       </c>
       <c r="C58" t="s">
         <v>154</v>
@@ -2145,10 +2151,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B59" s="3">
-        <v>46049</v>
+        <v>46051</v>
       </c>
       <c r="C59" t="s">
         <v>154</v>
@@ -2156,10 +2162,10 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B60" s="3">
-        <v>46044</v>
+        <v>46049</v>
       </c>
       <c r="C60" t="s">
         <v>154</v>
@@ -2167,78 +2173,89 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B61" s="3">
-        <v>46037</v>
+        <v>46044</v>
       </c>
       <c r="C61" t="s">
-        <v>297</v>
+        <v>154</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B62" s="3">
         <v>46037</v>
       </c>
       <c r="C62" t="s">
-        <v>10</v>
+        <v>297</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B63" s="3">
         <v>46037</v>
       </c>
       <c r="C63" t="s">
-        <v>298</v>
+        <v>10</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B64" s="3">
         <v>46037</v>
       </c>
       <c r="C64" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B65" s="3">
         <v>46037</v>
       </c>
       <c r="C65" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B66" s="3">
         <v>46037</v>
       </c>
       <c r="C66" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>339</v>
+      </c>
+      <c r="B67" s="3">
+        <v>46037</v>
+      </c>
+      <c r="C67" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
         <v>340</v>
       </c>
-      <c r="B67" s="3">
+      <c r="B68" s="3">
         <v>46035</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C68" t="s">
         <v>302</v>
       </c>
     </row>

</xml_diff>

<commit_message>
new Notification dgft and customs
</commit_message>
<xml_diff>
--- a/backend/PDF_DOC/CBIC/Notifications/Non-Tariff/Non-Tariff Notifications.xlsx
+++ b/backend/PDF_DOC/CBIC/Notifications/Non-Tariff/Non-Tariff Notifications.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2B23ADB-5BB6-4C62-B0EC-9858855B8BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB3FAEF-A1A6-4544-8695-21AF6EA1EA52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="383">
   <si>
     <t>Non-Tariff Notifications : 2024</t>
   </si>
@@ -1168,6 +1168,9 @@
   </si>
   <si>
     <t>Corrigendum to Tariff Notification No. 16/2026-Customs (NT) dated 2nd February, 2026</t>
+  </si>
+  <si>
+    <t>72/2026-Customs (NT)</t>
   </si>
 </sst>
 </file>
@@ -1535,7 +1538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.109375" customWidth="1"/>
@@ -1571,10 +1574,10 @@
     </row>
     <row r="6" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B6" s="10">
-        <v>46259</v>
+        <v>46265</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>154</v>
@@ -1582,10 +1585,10 @@
     </row>
     <row r="7" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B7" s="3">
-        <v>46248</v>
+        <v>46259</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>154</v>
@@ -1593,120 +1596,120 @@
     </row>
     <row r="8" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>378</v>
+      </c>
+      <c r="B8" s="3">
+        <v>46248</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>377</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B9" s="3">
         <v>46244</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>374</v>
-      </c>
-      <c r="B9" s="3">
-        <v>46234</v>
-      </c>
       <c r="C9" s="2" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B10" s="3">
         <v>46234</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>376</v>
+        <v>171</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>375</v>
+      </c>
+      <c r="B11" s="3">
+        <v>46234</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>372</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B12" s="3">
         <v>46223</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+    <row r="13" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>369</v>
-      </c>
-      <c r="B12" s="3">
-        <v>46219</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>371</v>
       </c>
       <c r="B13" s="3">
         <v>46219</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>163</v>
+        <v>370</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>371</v>
+      </c>
+      <c r="B14" s="3">
+        <v>46219</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>380</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B15" s="3">
         <v>46218</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
+      <c r="C15" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B16" s="3">
         <v>46206</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>368</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>365</v>
-      </c>
-      <c r="B16" s="3">
-        <v>46204</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>366</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B17" s="3">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>154</v>
+        <v>366</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B18" s="3">
-        <v>46202</v>
+        <v>46203</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>154</v>
@@ -1714,131 +1717,131 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B19" s="3">
-        <v>46195</v>
+        <v>46202</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>357</v>
+        <v>154</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="B20" s="3">
-        <v>46191</v>
+        <v>46195</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B21" s="3">
-        <v>46189</v>
+        <v>46191</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="B22" s="3">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>154</v>
+        <v>353</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>361</v>
+      </c>
+      <c r="B23" s="3">
+        <v>46188</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
         <v>354</v>
-      </c>
-      <c r="B23" s="3">
-        <v>46184</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>362</v>
       </c>
       <c r="B24" s="3">
         <v>46184</v>
       </c>
       <c r="C24" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>362</v>
+      </c>
+      <c r="B25" s="3">
+        <v>46184</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>355</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>351</v>
-      </c>
-      <c r="B25" s="3">
-        <v>46182</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="B26" s="3">
-        <v>46178</v>
+        <v>46182</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B27" s="3">
         <v>46178</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>344</v>
+      </c>
+      <c r="B28" s="3">
+        <v>46178</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>345</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>346</v>
-      </c>
-      <c r="B28" s="3">
-        <v>46171</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B29" s="3">
-        <v>46161</v>
+        <v>46171</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B30" s="3">
-        <v>46157</v>
+        <v>46161</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>154</v>
@@ -1846,10 +1849,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B31" s="3">
-        <v>46150</v>
+        <v>46157</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>154</v>
@@ -1857,208 +1860,208 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="B32" s="3">
-        <v>46148</v>
+        <v>46150</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>341</v>
+        <v>154</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>320</v>
+        <v>350</v>
       </c>
       <c r="B33" s="3">
-        <v>46142</v>
+        <v>46148</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>154</v>
+        <v>341</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B34" s="3">
-        <v>46136</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>163</v>
+        <v>46142</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>318</v>
+      </c>
+      <c r="B35" s="3">
+        <v>46136</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
         <v>321</v>
       </c>
-      <c r="B35" s="3">
+      <c r="B36" s="3">
         <v>46132</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C36" s="8" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
+    <row r="37" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
         <v>316</v>
       </c>
-      <c r="B36" s="3">
+      <c r="B37" s="3">
         <v>46128</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C37" s="2" t="s">
         <v>317</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>322</v>
-      </c>
-      <c r="B37" s="3">
-        <v>46127</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B38" s="3">
-        <v>46118</v>
+        <v>46127</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>315</v>
+        <v>154</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B39" s="3">
-        <v>46114</v>
+        <v>46118</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>154</v>
+        <v>315</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>191</v>
+        <v>324</v>
       </c>
       <c r="B40" s="3">
-        <v>46112</v>
+        <v>46114</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>311</v>
+        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B41" s="3">
         <v>46112</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>325</v>
+        <v>192</v>
       </c>
       <c r="B42" s="3">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>171</v>
+        <v>312</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B43" s="3">
         <v>46111</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>313</v>
+        <v>171</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B44" s="3">
-        <v>46105</v>
+        <v>46111</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B45" s="3">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B46" s="3">
         <v>46101</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>171</v>
+        <v>309</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B47" s="3">
-        <v>46100</v>
+        <v>46101</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>265</v>
+        <v>330</v>
       </c>
       <c r="B48" s="3">
-        <v>46097</v>
+        <v>46100</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>310</v>
+        <v>154</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B49" s="3">
-        <v>46094</v>
+        <v>46097</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>154</v>
+        <v>310</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>201</v>
+        <v>266</v>
       </c>
       <c r="B50" s="3">
-        <v>46077</v>
+        <v>46094</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>154</v>
@@ -2066,43 +2069,43 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
+        <v>201</v>
+      </c>
+      <c r="B51" s="3">
+        <v>46077</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
         <v>303</v>
       </c>
-      <c r="B51" s="3">
+      <c r="B52" s="3">
         <v>46071</v>
       </c>
-      <c r="C51" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
+      <c r="C52" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>304</v>
       </c>
-      <c r="B52" s="3">
+      <c r="B53" s="3">
         <v>46069</v>
       </c>
-      <c r="C52" s="2" t="s">
+      <c r="C53" s="2" t="s">
         <v>176</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>305</v>
-      </c>
-      <c r="B53" s="3">
-        <v>46066</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B54" s="3">
-        <v>46059</v>
+        <v>46066</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>154</v>
@@ -2110,10 +2113,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B55" s="3">
-        <v>46058</v>
+        <v>46059</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>154</v>
@@ -2121,98 +2124,98 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
+        <v>307</v>
+      </c>
+      <c r="B56" s="3">
+        <v>46058</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
         <v>308</v>
-      </c>
-      <c r="B56" s="3">
-        <v>46056</v>
-      </c>
-      <c r="C56" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A57" s="2" t="s">
-        <v>381</v>
       </c>
       <c r="B57" s="3">
         <v>46056</v>
       </c>
       <c r="C57" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A58" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="B58" s="3">
+        <v>46056</v>
+      </c>
+      <c r="C58" t="s">
         <v>286</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>287</v>
-      </c>
-      <c r="B58" s="3">
-        <v>46055</v>
-      </c>
-      <c r="C58" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B59" s="3">
-        <v>46054</v>
+        <v>46055</v>
       </c>
       <c r="C59" t="s">
-        <v>289</v>
+        <v>154</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B60" s="3">
         <v>46054</v>
       </c>
       <c r="C60" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B61" s="3">
         <v>46054</v>
       </c>
       <c r="C61" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B62" s="3">
         <v>46054</v>
       </c>
       <c r="C62" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B63" s="3">
-        <v>46052</v>
+        <v>46054</v>
       </c>
       <c r="C63" t="s">
-        <v>154</v>
+        <v>295</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>331</v>
+        <v>296</v>
       </c>
       <c r="B64" s="3">
-        <v>46051</v>
+        <v>46052</v>
       </c>
       <c r="C64" t="s">
         <v>154</v>
@@ -2220,10 +2223,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B65" s="3">
-        <v>46049</v>
+        <v>46051</v>
       </c>
       <c r="C65" t="s">
         <v>154</v>
@@ -2231,10 +2234,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="B66" s="3">
-        <v>46044</v>
+        <v>46049</v>
       </c>
       <c r="C66" t="s">
         <v>154</v>
@@ -2242,78 +2245,89 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="B67" s="3">
-        <v>46037</v>
+        <v>46044</v>
       </c>
       <c r="C67" t="s">
-        <v>297</v>
+        <v>154</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="B68" s="3">
         <v>46037</v>
       </c>
       <c r="C68" t="s">
-        <v>10</v>
+        <v>297</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="B69" s="3">
         <v>46037</v>
       </c>
       <c r="C69" t="s">
-        <v>298</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B70" s="3">
         <v>46037</v>
       </c>
       <c r="C70" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B71" s="3">
         <v>46037</v>
       </c>
       <c r="C71" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B72" s="3">
         <v>46037</v>
       </c>
       <c r="C72" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
+        <v>339</v>
+      </c>
+      <c r="B73" s="3">
+        <v>46037</v>
+      </c>
+      <c r="C73" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
         <v>340</v>
       </c>
-      <c r="B73" s="3">
+      <c r="B74" s="3">
         <v>46035</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C74" t="s">
         <v>302</v>
       </c>
     </row>

</xml_diff>